<commit_message>
all maps and final codes
</commit_message>
<xml_diff>
--- a/data/controles_results/dif_medias/controls_vars/difmedias_controles_baselines_fixed_2018_T1.xlsx
+++ b/data/controles_results/dif_medias/controls_vars/difmedias_controles_baselines_fixed_2018_T1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="224" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="168" uniqueCount="77">
   <si>
     <t/>
   </si>
@@ -24,12 +24,6 @@
     <t>poblacion_urbana_2009</t>
   </si>
   <si>
-    <t>poblacion_por_localidad_2005</t>
-  </si>
-  <si>
-    <t>poblacion_2005</t>
-  </si>
-  <si>
     <t>personas_por_localidad_2007</t>
   </si>
   <si>
@@ -48,12 +42,6 @@
     <t>estrato_mean</t>
   </si>
   <si>
-    <t>densidad_urbana_2009</t>
-  </si>
-  <si>
-    <t>area_urbana_2009</t>
-  </si>
-  <si>
     <t>acceso_transmi</t>
   </si>
   <si>
@@ -63,7 +51,7 @@
     <t>accesibilidad_arterial_dummy</t>
   </si>
   <si>
-    <t xml:space="preserve">If the table includes missing values (.n, .o, .v etc.) see the Missing values section in the help file for the Stata command iebaltab for definitions of these values. Significance: ***=.01, **=.05, *=.1. Full user input as written by user: [iebaltab poblacion_urbana_2009 poblacion_por_localidad_2005 poblacion_2005 personas_por_localidad_2007 personas_por_hogar_2007_localida num_est_transmi icv_2007_localidad gasto_promedio_mensual_2007_loca estrato_mean densidad_urbana_2009 area_urbana_2009 acceso_transmi accesibilidad_arterial accesibilidad_arterial_dummy, groupvar(dummy_oxxo) control(0) savexlsx(difmedias_controles_baselines_fixed_2018_T1) replace] </t>
+    <t xml:space="preserve">If the table includes missing values (.n, .o, .v etc.) see the Missing values section in the help file for the Stata command iebaltab for definitions of these values. Significance: ***=.01, **=.05, *=.1. Full user input as written by user: [iebaltab poblacion_urbana_2009 personas_por_localidad_2007 personas_por_hogar_2007_localida num_est_transmi icv_2007_localidad gasto_promedio_mensual_2007_loca estrato_mean acceso_transmi accesibilidad_arterial accesibilidad_arterial_dummy, groupvar(dummy_oxxo) control(0) savexlsx(difmedias_controles_baselines_fixed_2018_T1) replace] </t>
   </si>
   <si>
     <t>N</t>
@@ -84,28 +72,16 @@
     <t>Mean/(SE)</t>
   </si>
   <si>
-    <t>64370.418</t>
-  </si>
-  <si>
-    <t>(5891.527)</t>
-  </si>
-  <si>
-    <t>485.996</t>
-  </si>
-  <si>
-    <t>(30.427)</t>
-  </si>
-  <si>
-    <t>60480.451</t>
-  </si>
-  <si>
-    <t>(5536.453)</t>
-  </si>
-  <si>
-    <t>501.863</t>
-  </si>
-  <si>
-    <t>(31.911)</t>
+    <t>6.16e+05</t>
+  </si>
+  <si>
+    <t>(75840.889)</t>
+  </si>
+  <si>
+    <t>501.155</t>
+  </si>
+  <si>
+    <t>(31.953)</t>
   </si>
   <si>
     <t>3.572</t>
@@ -114,10 +90,10 @@
     <t>(0.041)</t>
   </si>
   <si>
-    <t>1.579</t>
-  </si>
-  <si>
-    <t>(0.201)</t>
+    <t>11.560</t>
+  </si>
+  <si>
+    <t>(1.655)</t>
   </si>
   <si>
     <t>88.933</t>
@@ -138,25 +114,16 @@
     <t>(0.117)</t>
   </si>
   <si>
-    <t>2.88e+11</t>
-  </si>
-  <si>
-    <t>(2.56e+10)</t>
-  </si>
-  <si>
-    <t>3.54e+11</t>
-  </si>
-  <si>
-    <t>(2.17e+10)</t>
-  </si>
-  <si>
-    <t>0.477</t>
-  </si>
-  <si>
-    <t>4.282</t>
-  </si>
-  <si>
-    <t>(0.244)</t>
+    <t>3.571</t>
+  </si>
+  <si>
+    <t>(0.395)</t>
+  </si>
+  <si>
+    <t>34.571</t>
+  </si>
+  <si>
+    <t>(3.049)</t>
   </si>
   <si>
     <t>0.978</t>
@@ -174,22 +141,10 @@
     <t>1</t>
   </si>
   <si>
-    <t>61128.174</t>
-  </si>
-  <si>
-    <t>(9867.834)</t>
-  </si>
-  <si>
-    <t>456.961</t>
-  </si>
-  <si>
-    <t>(71.156)</t>
-  </si>
-  <si>
-    <t>59507.696</t>
-  </si>
-  <si>
-    <t>(9328.271)</t>
+    <t>6.57e+05</t>
+  </si>
+  <si>
+    <t>(1.32e+05)</t>
   </si>
   <si>
     <t>474.421</t>
@@ -204,10 +159,10 @@
     <t>(0.079)</t>
   </si>
   <si>
-    <t>3.844</t>
-  </si>
-  <si>
-    <t>(0.544)</t>
+    <t>35.087</t>
+  </si>
+  <si>
+    <t>(6.038)</t>
   </si>
   <si>
     <t>91.483</t>
@@ -228,28 +183,16 @@
     <t>(0.183)</t>
   </si>
   <si>
-    <t>2.96e+11</t>
-  </si>
-  <si>
-    <t>(5.27e+10)</t>
-  </si>
-  <si>
-    <t>3.58e+11</t>
-  </si>
-  <si>
-    <t>(4.01e+10)</t>
-  </si>
-  <si>
-    <t>0.809</t>
-  </si>
-  <si>
-    <t>(0.060)</t>
-  </si>
-  <si>
-    <t>6.026</t>
-  </si>
-  <si>
-    <t>(0.586)</t>
+    <t>7.391</t>
+  </si>
+  <si>
+    <t>(0.857)</t>
+  </si>
+  <si>
+    <t>49.826</t>
+  </si>
+  <si>
+    <t>(4.839)</t>
   </si>
   <si>
     <t>1.000</t>
@@ -273,22 +216,16 @@
     <t>Mean difference</t>
   </si>
   <si>
-    <t>-3242.244</t>
-  </si>
-  <si>
-    <t>-29.034</t>
-  </si>
-  <si>
-    <t>-972.755</t>
-  </si>
-  <si>
-    <t>-27.442</t>
+    <t>41250.355</t>
+  </si>
+  <si>
+    <t>-26.735</t>
   </si>
   <si>
     <t>-0.314***</t>
   </si>
   <si>
-    <t>2.265***</t>
+    <t>23.527***</t>
   </si>
   <si>
     <t>2.551***</t>
@@ -300,16 +237,10 @@
     <t>0.812***</t>
   </si>
   <si>
-    <t>8.59e+09</t>
-  </si>
-  <si>
-    <t>3.57e+09</t>
-  </si>
-  <si>
-    <t>0.333***</t>
-  </si>
-  <si>
-    <t>1.744***</t>
+    <t>3.820***</t>
+  </si>
+  <si>
+    <t>15.255**</t>
   </si>
   <si>
     <t>0.022</t>
@@ -356,7 +287,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -367,19 +298,19 @@
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
       </c>
       <c r="E1" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="F1" t="s">
         <v>0</v>
       </c>
       <c r="G1" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2">
@@ -390,19 +321,19 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D2" t="s">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="F2" t="s">
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>84</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3">
@@ -410,22 +341,22 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G3" t="s">
-        <v>85</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4">
@@ -433,22 +364,22 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="F4" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="G4" t="s">
-        <v>86</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5">
@@ -459,13 +390,13 @@
         <v>0</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
         <v>0</v>
       </c>
       <c r="E5" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="F5" t="s">
         <v>0</v>
@@ -479,22 +410,22 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="G6" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7">
@@ -505,13 +436,13 @@
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="D7" t="s">
         <v>0</v>
       </c>
       <c r="E7" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="F7" t="s">
         <v>0</v>
@@ -525,22 +456,22 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="F8" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="G8" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9">
@@ -551,13 +482,13 @@
         <v>0</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D9" t="s">
         <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="F9" t="s">
         <v>0</v>
@@ -571,22 +502,22 @@
         <v>5</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="F10" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="G10" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11">
@@ -597,13 +528,13 @@
         <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D11" t="s">
         <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="F11" t="s">
         <v>0</v>
@@ -617,22 +548,22 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12" t="s">
         <v>50</v>
       </c>
-      <c r="E12" t="s">
-        <v>61</v>
-      </c>
       <c r="F12" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="G12" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13">
@@ -643,13 +574,13 @@
         <v>0</v>
       </c>
       <c r="C13" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D13" t="s">
         <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
         <v>0</v>
@@ -663,22 +594,22 @@
         <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="E14" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="G14" t="s">
-        <v>91</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15">
@@ -689,13 +620,13 @@
         <v>0</v>
       </c>
       <c r="C15" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="D15" t="s">
         <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="F15" t="s">
         <v>0</v>
@@ -709,22 +640,22 @@
         <v>8</v>
       </c>
       <c r="B16" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="E16" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="G16" t="s">
-        <v>92</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17">
@@ -735,13 +666,13 @@
         <v>0</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D17" t="s">
         <v>0</v>
       </c>
       <c r="E17" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="F17" t="s">
         <v>0</v>
@@ -755,22 +686,22 @@
         <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D18" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="F18" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="G18" t="s">
-        <v>93</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19">
@@ -781,13 +712,13 @@
         <v>0</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D19" t="s">
         <v>0</v>
       </c>
       <c r="E19" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="F19" t="s">
         <v>0</v>
@@ -801,22 +732,22 @@
         <v>10</v>
       </c>
       <c r="B20" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="D20" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="E20" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="F20" t="s">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="G20" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21">
@@ -827,13 +758,13 @@
         <v>0</v>
       </c>
       <c r="C21" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D21" t="s">
         <v>0</v>
       </c>
       <c r="E21" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="F21" t="s">
         <v>0</v>
@@ -847,22 +778,22 @@
         <v>11</v>
       </c>
       <c r="B22" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="D22" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="E22" t="s">
-        <v>71</v>
+        <v>60</v>
       </c>
       <c r="F22" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="G22" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23">
@@ -873,13 +804,13 @@
         <v>0</v>
       </c>
       <c r="C23" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D23" t="s">
         <v>0</v>
       </c>
       <c r="E23" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="F23" t="s">
         <v>0</v>
@@ -893,205 +824,21 @@
         <v>12</v>
       </c>
       <c r="B24" t="s">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="C24" t="s">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="D24" t="s">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="F24" t="s">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="G24" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s">
-        <v>0</v>
-      </c>
-      <c r="B25" t="s">
-        <v>0</v>
-      </c>
-      <c r="C25" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25" t="s">
-        <v>0</v>
-      </c>
-      <c r="E25" t="s">
-        <v>74</v>
-      </c>
-      <c r="F25" t="s">
-        <v>0</v>
-      </c>
-      <c r="G25" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s">
-        <v>13</v>
-      </c>
-      <c r="B26" t="s">
-        <v>18</v>
-      </c>
-      <c r="C26" t="s">
-        <v>45</v>
-      </c>
-      <c r="D26" t="s">
-        <v>50</v>
-      </c>
-      <c r="E26" t="s">
-        <v>75</v>
-      </c>
-      <c r="F26" t="s">
-        <v>81</v>
-      </c>
-      <c r="G26" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="s">
-        <v>0</v>
-      </c>
-      <c r="B27" t="s">
-        <v>0</v>
-      </c>
-      <c r="C27" t="s">
-        <v>32</v>
-      </c>
-      <c r="D27" t="s">
-        <v>0</v>
-      </c>
-      <c r="E27" t="s">
-        <v>76</v>
-      </c>
-      <c r="F27" t="s">
-        <v>0</v>
-      </c>
-      <c r="G27" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B28" t="s">
-        <v>18</v>
-      </c>
-      <c r="C28" t="s">
-        <v>46</v>
-      </c>
-      <c r="D28" t="s">
-        <v>50</v>
-      </c>
-      <c r="E28" t="s">
-        <v>77</v>
-      </c>
-      <c r="F28" t="s">
-        <v>81</v>
-      </c>
-      <c r="G28" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="s">
-        <v>0</v>
-      </c>
-      <c r="B29" t="s">
-        <v>0</v>
-      </c>
-      <c r="C29" t="s">
-        <v>47</v>
-      </c>
-      <c r="D29" t="s">
-        <v>0</v>
-      </c>
-      <c r="E29" t="s">
-        <v>78</v>
-      </c>
-      <c r="F29" t="s">
-        <v>0</v>
-      </c>
-      <c r="G29" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30" t="s">
-        <v>18</v>
-      </c>
-      <c r="C30" t="s">
-        <v>48</v>
-      </c>
-      <c r="D30" t="s">
-        <v>50</v>
-      </c>
-      <c r="E30" t="s">
-        <v>79</v>
-      </c>
-      <c r="F30" t="s">
-        <v>81</v>
-      </c>
-      <c r="G30" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="s">
-        <v>0</v>
-      </c>
-      <c r="B31" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" t="s">
-        <v>49</v>
-      </c>
-      <c r="D31" t="s">
-        <v>0</v>
-      </c>
-      <c r="E31" t="s">
-        <v>80</v>
-      </c>
-      <c r="F31" t="s">
-        <v>0</v>
-      </c>
-      <c r="G31" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="s">
-        <v>16</v>
-      </c>
-      <c r="B32" t="s">
-        <v>0</v>
-      </c>
-      <c r="C32" t="s">
-        <v>0</v>
-      </c>
-      <c r="D32" t="s">
-        <v>0</v>
-      </c>
-      <c r="E32" t="s">
-        <v>0</v>
-      </c>
-      <c r="F32" t="s">
-        <v>0</v>
-      </c>
-      <c r="G32" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>